<commit_message>
PAUSED (task255): loop 2 built and gated, stage 4 readers and judge running
The coverage-group severity build: 281 checks, the independent verifier, byte-identical rebuilds,
figures_check 93, precut 51, leak.py REVIEW, heart WARN, surface PASS, pair ceiling 35.4. The ask
layer is re-sited (a member leaving on 31 December 2026, re-declarations on adopted budgets,
vehicles transferred between members). Expected occurrences are graded to one decimal. Resume from
pipeline.json: score the two readers, take the judge's verdict, fix, reship.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Es2YJxT597uNAuNJZNdYR4
</commit_message>
<xml_diff>
--- a/task255/golden/retention_2027.xlsx
+++ b/task255/golden/retention_2027.xlsx
@@ -24,15 +24,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
   <si>
     <t>Fallowmere Intergovernmental Risk Pool</t>
   </si>
   <si>
-    <t>Keep the first $4,000,000 of each 2027 liability occurrence: the lowest quoted attachment the pool expects its 2027 occurrences to exceed once or less (0.74)</t>
-  </si>
-  <si>
-    <t>Risk financing policy 4.1 to 5.1; expected occurrences from the actuary's 228.7 above $25,000 and the ground-up severity curve at 2027 cost; premiums from the broker's indications of October 2, 2026.</t>
+    <t>Keep the first $4,000,000 of each 2027 liability occurrence: the lowest quoted attachment the pool expects its 2027 occurrences to exceed once or less (0.8)</t>
+  </si>
+  <si>
+    <t>Risk financing policy 4.1 to 5.1; expected occurrences from the actuary's 84.7 law enforcement and 364.7 other occurrences above $25,000, each carried by its own ground-up severity at 2027 cost; premiums from the broker's indications of October 2, 2026.</t>
   </si>
   <si>
     <t>Attachment per occurrence</t>
@@ -59,34 +59,40 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>Severity curve (lognormal, cost from the first dollar at 2027 cost)</t>
-  </si>
-  <si>
-    <t>log mean 10.18, log standard deviation 1.71</t>
+    <t>Severity, law enforcement liability (lognormal, from the first dollar at 2027 cost)</t>
+  </si>
+  <si>
+    <t>log mean 8.52, log standard deviation 2.37; 314 occurrences, 25 of them stopped at the retention</t>
+  </si>
+  <si>
+    <t>Severity, general, auto, public officials' and employment practices liability</t>
+  </si>
+  <si>
+    <t>log mean 9.89, log standard deviation 1.14; 757 occurrences, 0 of them stopped at the retention</t>
   </si>
   <si>
     <t>Fitted to</t>
   </si>
   <si>
-    <t>820 occurrences of accident years 2014 to 2021 in the pool's record (800 closed, 20 suits still open with the pool's layer paid), 108 of them stopped at the retention</t>
+    <t>1071 occurrences of accident years 2014 to 2021 in the pool's record (1063 closed, 8 suits still open with the pool's layer paid)</t>
   </si>
   <si>
     <t>How the record enters the fit</t>
   </si>
   <si>
-    <t>each occurrence truncated at its member's deductible and, where it reached the pool's retention, censored there; costs, deductibles and retentions at 2027 cost by the claim cost index</t>
+    <t>each occurrence truncated at its member's deductible and, where it reached the pool's retention, censored there; costs, deductibles and retentions at 2027 cost by the claim cost index; one curve over every coverage part does not fit the record (likelihood ratio 158 on two degrees of freedom)</t>
   </si>
   <si>
     <t>Runner-up</t>
   </si>
   <si>
-    <t>$3,000,000: 1.25 expected occurrences above it, more than the policy's one</t>
+    <t>$3,000,000: 1.2 expected occurrences above it, more than the policy's one</t>
   </si>
   <si>
     <t>Rated exposure</t>
   </si>
   <si>
-    <t>2027 operating expenditures of $5,668,433,420 as declared; 5,649 units on the vehicle schedules at September 30, 2026 (sheet Rated exposure)</t>
+    <t>2027 operating expenditures of $5,705,912,536 as declared; 5,637 units on the vehicle schedules at September 30, 2026 (sheet Rated exposure)</t>
   </si>
   <si>
     <t>Exposure the 2027 indications are rated on, by member class</t>
@@ -134,16 +140,16 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Prepared for the Board of Trustees' meeting of November 18, 2026, from the claims records at September 30, 2026, the actuary's study of October 9, 2026 and the broker's indications of October 2, 2026.</t>
+    <t>Prepared for the executive director's 2027 budget proposal, from the claims records at September 30, 2026, the actuary's study of October 9, 2026 and the broker's indications of October 2, 2026.</t>
   </si>
   <si>
     <t>Cost of an occurrence: from its first dollar, damages and defense together, whoever pays (policy 2.2). Attachments are from the first dollar, inclusive of the member's deductible (policy 2.3).</t>
   </si>
   <si>
-    <t>The pool's record holds an occurrence only once its member's payments reached the deductible in force on the date of the occurrence, and holds its cost only up to the pool's retention ($250,000 for 2014 to 2017, $500,000 from 2018); the curve is fitted to that record as it came to exist.</t>
-  </si>
-  <si>
-    <t>Expected occurrences above an attachment: 228.7 times the curve's probability of a cost above the attachment over its probability of a cost above $25,000 (policy 4.3). Shown to two decimals; compared unrounded.</t>
+    <t>The pool's record holds an occurrence only once its member's payments reached the deductible in force on the date of the occurrence, and holds its cost only up to the pool's retention ($500,000 for 2014 to 2017, $1,000,000 from 2018); severity is fitted to that record as it came to exist.</t>
+  </si>
+  <si>
+    <t>Expected occurrences above an attachment: the actuary's 84.7 law enforcement occurrences above $25,000 times that severity's probability of a cost above the attachment given a cost above $25,000, plus the same for the 364.7 other occurrences (policy 4.3, Exhibit 6). Shown to one decimal; compared unrounded.</t>
   </si>
   <si>
     <t>Premiums: the indicated rates applied to the declared 2027 operating expenditures and the scheduled units; annual, before the Washington surplus lines tax and stamping fee; rounded to the dollar.</t>
@@ -159,10 +165,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
-    <numFmt numFmtId="165" formatCode="$0.0000"/>
-    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="$0.0000"/>
+    <numFmt numFmtId="167" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -254,19 +261,19 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -575,7 +582,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B798F5D-9355-556D-A21E-16F5F5D7355A}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
@@ -626,7 +633,7 @@
         <v>1000000</v>
       </c>
       <c r="B6" s="6">
-        <v>7.46</v>
+        <v>4.6</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>9</v>
@@ -638,7 +645,7 @@
         <v>71.40000000000001</v>
       </c>
       <c r="F6" s="5">
-        <v>1770565</v>
+        <v>1778748</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -646,7 +653,7 @@
         <v>1500000</v>
       </c>
       <c r="B7" s="6">
-        <v>4.03</v>
+        <v>2.8</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>9</v>
@@ -658,7 +665,7 @@
         <v>56.85</v>
       </c>
       <c r="F7" s="5">
-        <v>1414020</v>
+        <v>1420563</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -666,7 +673,7 @@
         <v>2000000</v>
       </c>
       <c r="B8" s="6">
-        <v>2.53</v>
+        <v>2</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>9</v>
@@ -678,7 +685,7 @@
         <v>48.65</v>
       </c>
       <c r="F8" s="5">
-        <v>1180073</v>
+        <v>1185474</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -686,7 +693,7 @@
         <v>2500000</v>
       </c>
       <c r="B9" s="6">
-        <v>1.73</v>
+        <v>1.5</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>9</v>
@@ -698,7 +705,7 @@
         <v>41.2</v>
       </c>
       <c r="F9" s="5">
-        <v>1017817</v>
+        <v>1022513</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -706,7 +713,7 @@
         <v>3000000</v>
       </c>
       <c r="B10" s="6">
-        <v>1.25</v>
+        <v>1.2</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>9</v>
@@ -718,7 +725,7 @@
         <v>36.3</v>
       </c>
       <c r="F10" s="5">
-        <v>881870</v>
+        <v>885909</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -726,7 +733,7 @@
         <v>4000000</v>
       </c>
       <c r="B11" s="11">
-        <v>0.74</v>
+        <v>0.8</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>10</v>
@@ -738,7 +745,7 @@
         <v>31.75</v>
       </c>
       <c r="F11" s="10">
-        <v>735429</v>
+        <v>738725</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -746,7 +753,7 @@
         <v>5000000</v>
       </c>
       <c r="B12" s="6">
-        <v>0.48</v>
+        <v>0.6</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>10</v>
@@ -758,7 +765,7 @@
         <v>31.75</v>
       </c>
       <c r="F12" s="5">
-        <v>641333</v>
+        <v>644007</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -799,6 +806,14 @@
       </c>
       <c r="B18" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -819,138 +834,138 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B5">
         <v>33</v>
       </c>
       <c r="C5" s="16">
-        <v>4992928</v>
+        <v>5043163</v>
       </c>
       <c r="D5" s="16">
-        <v>4207</v>
+        <v>4202</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B6">
         <v>9</v>
       </c>
       <c r="C6" s="16">
-        <v>121458</v>
+        <v>120787</v>
       </c>
       <c r="D6" s="16">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C7" s="16">
-        <v>126705</v>
+        <v>121297</v>
       </c>
       <c r="D7" s="16">
-        <v>241</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B8">
         <v>3</v>
       </c>
       <c r="C8" s="16">
-        <v>141394</v>
+        <v>136810</v>
       </c>
       <c r="D8" s="16">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B9">
         <v>2</v>
       </c>
       <c r="C9" s="16">
-        <v>218248</v>
+        <v>217085</v>
       </c>
       <c r="D9" s="16">
-        <v>541</v>
+        <v>542</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B10">
         <v>4</v>
       </c>
       <c r="C10" s="16">
-        <v>50231</v>
+        <v>49785</v>
       </c>
       <c r="D10" s="16">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B11">
         <v>3</v>
       </c>
       <c r="C11" s="16">
-        <v>17470</v>
+        <v>16985</v>
       </c>
       <c r="D11" s="16">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B12" s="15">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C12" s="17">
-        <v>5668433</v>
+        <v>5705913</v>
       </c>
       <c r="D12" s="17">
-        <v>5649</v>
+        <v>5637</v>
       </c>
     </row>
   </sheetData>
@@ -968,42 +983,42 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PAUSED (task255): loop 2 asks follow the severity construction, stage 4 round 2 running
Round 1 readers both missed the call at USD 2.0 million but solved every exposure figure, so the
premium and class-exposure asks are replaced by each quoted layer's expected 2027 losses; anchors
85.0 and 375.0 keep every count and layer loss clear of its rounding edge under the five-part fit;
quotes rescaled by one market factor; same-day occurrences separated. 282 checks, verify,
byte-identical rebuilds, precut 51, leak.py REVIEW, pair ceiling 56.0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Es2YJxT597uNAuNJZNdYR4
</commit_message>
<xml_diff>
--- a/task255/golden/retention_2027.xlsx
+++ b/task255/golden/retention_2027.xlsx
@@ -8,8 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Retention 2027" sheetId="1" r:id="rId1"/>
-    <sheet name="Rated exposure" sheetId="2" r:id="rId2"/>
-    <sheet name="Notes" sheetId="3" r:id="rId3"/>
+    <sheet name="Notes" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Retention 2027'!$5:$5</definedName>
@@ -24,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
   <si>
     <t>Fallowmere Intergovernmental Risk Pool</t>
   </si>
@@ -32,7 +31,7 @@
     <t>Keep the first $4,000,000 of each 2027 liability occurrence: the lowest quoted attachment the pool expects its 2027 occurrences to exceed once or less (0.8)</t>
   </si>
   <si>
-    <t>Risk financing policy 4.1 to 5.1; expected occurrences from the actuary's 84.7 law enforcement and 364.7 other occurrences above $25,000, each carried by its own ground-up severity at 2027 cost; premiums from the broker's indications of October 2, 2026.</t>
+    <t>Risk financing policy 4.1 to 5.1; expected occurrences from the actuary's 85.0 law enforcement and 375.0 other occurrences above $25,000, each carried by its own ground-up severity at 2027 cost; layers of $10,000,000 above each attachment quoted by the broker on October 2, 2026.</t>
   </si>
   <si>
     <t>Attachment per occurrence</t>
@@ -44,13 +43,7 @@
     <t>Within the policy (one or fewer)</t>
   </si>
   <si>
-    <t>Rate per $1,000 of operating expenditures</t>
-  </si>
-  <si>
-    <t>Rate per scheduled unit</t>
-  </si>
-  <si>
-    <t>2027 premium</t>
+    <t>Expected 2027 losses to the $10,000,000 layer</t>
   </si>
   <si>
     <t>No</t>
@@ -89,54 +82,6 @@
     <t>$3,000,000: 1.2 expected occurrences above it, more than the policy's one</t>
   </si>
   <si>
-    <t>Rated exposure</t>
-  </si>
-  <si>
-    <t>2027 operating expenditures of $5,705,912,536 as declared; 5,637 units on the vehicle schedules at September 30, 2026 (sheet Rated exposure)</t>
-  </si>
-  <si>
-    <t>Exposure the 2027 indications are rated on, by member class</t>
-  </si>
-  <si>
-    <t>Operating expenditures: each member's 2027 total as declared for the renewal (once per member). Vehicles: units on the members' schedules at September 30, 2026, one per vehicle.</t>
-  </si>
-  <si>
-    <t>Member class</t>
-  </si>
-  <si>
-    <t>Members</t>
-  </si>
-  <si>
-    <t>2027 operating expenditures ($000)</t>
-  </si>
-  <si>
-    <t>Scheduled vehicles</t>
-  </si>
-  <si>
-    <t>City</t>
-  </si>
-  <si>
-    <t>Fire district</t>
-  </si>
-  <si>
-    <t>Water-sewer district</t>
-  </si>
-  <si>
-    <t>Port district</t>
-  </si>
-  <si>
-    <t>Transit authority</t>
-  </si>
-  <si>
-    <t>Park and recreation district</t>
-  </si>
-  <si>
-    <t>Library district</t>
-  </si>
-  <si>
-    <t>All members</t>
-  </si>
-  <si>
     <t>Notes</t>
   </si>
   <si>
@@ -149,27 +94,19 @@
     <t>The pool's record holds an occurrence only once its member's payments reached the deductible in force on the date of the occurrence, and holds its cost only up to the pool's retention ($500,000 for 2014 to 2017, $1,000,000 from 2018); severity is fitted to that record as it came to exist.</t>
   </si>
   <si>
-    <t>Expected occurrences above an attachment: the actuary's 84.7 law enforcement occurrences above $25,000 times that severity's probability of a cost above the attachment given a cost above $25,000, plus the same for the 364.7 other occurrences (policy 4.3, Exhibit 6). Shown to one decimal; compared unrounded.</t>
-  </si>
-  <si>
-    <t>Premiums: the indicated rates applied to the declared 2027 operating expenditures and the scheduled units; annual, before the Washington surplus lines tax and stamping fee; rounded to the dollar.</t>
-  </si>
-  <si>
-    <t>Vehicles loaded from the fleet consortium's lists on March 4, 2024 carry the consortium's asset numbers; a vehicle counts once, under the latest number added for it.</t>
-  </si>
-  <si>
-    <t>Rated exposure: each class's operating expenditures are rounded to the thousand on their own and the total from the unrounded sum, so the classes can differ from the total by a thousand dollars.</t>
+    <t>Expected occurrences above an attachment: the actuary's 85.0 law enforcement occurrences above $25,000 times that severity's probability of a cost above the attachment given a cost above $25,000, plus the same for the 375.0 other occurrences (policy 4.3, Exhibit 6). Shown to one decimal; compared unrounded.</t>
+  </si>
+  <si>
+    <t>Expected losses to a layer: for each coverage group, its expected 2027 occurrences above $25,000 times the expected cost above the attachment, up to the $10,000,000 limit, of an occurrence costing more than $25,000 on that group's severity; rounded to the nearest hundred thousand dollars.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="$0.0000"/>
-    <numFmt numFmtId="167" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -252,7 +189,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -265,18 +202,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -582,33 +513,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B798F5D-9355-556D-A21E-16F5F5D7355A}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
     <col min="2" max="2" width="20.7109375" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" customWidth="1"/>
+    <col min="4" max="4" width="24.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="44" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="44" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
@@ -621,14 +550,8 @@
       <c r="D5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>1000000</v>
       </c>
@@ -636,19 +559,13 @@
         <v>4.6</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="8">
-        <v>0.2412</v>
-      </c>
-      <c r="E6" s="9">
-        <v>71.40000000000001</v>
-      </c>
-      <c r="F6" s="5">
-        <v>1778748</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="D6" s="5">
+        <v>8300000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>1500000</v>
       </c>
@@ -656,19 +573,13 @@
         <v>2.8</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="8">
-        <v>0.1928</v>
-      </c>
-      <c r="E7" s="9">
-        <v>56.85</v>
-      </c>
-      <c r="F7" s="5">
-        <v>1420563</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="D7" s="5">
+        <v>6600000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>2000000</v>
       </c>
@@ -676,19 +587,13 @@
         <v>2</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="8">
-        <v>0.1597</v>
-      </c>
-      <c r="E8" s="9">
-        <v>48.65</v>
-      </c>
-      <c r="F8" s="5">
-        <v>1185474</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="D8" s="5">
+        <v>5500000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>2500000</v>
       </c>
@@ -696,19 +601,13 @@
         <v>1.5</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="8">
-        <v>0.1385</v>
-      </c>
-      <c r="E9" s="9">
-        <v>41.2</v>
-      </c>
-      <c r="F9" s="5">
-        <v>1022513</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="D9" s="5">
+        <v>4700000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>3000000</v>
       </c>
@@ -716,39 +615,27 @@
         <v>1.2</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="8">
-        <v>0.1194</v>
-      </c>
-      <c r="E10" s="9">
-        <v>36.3</v>
-      </c>
-      <c r="F10" s="5">
-        <v>885909</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="10">
+        <v>7</v>
+      </c>
+      <c r="D10" s="5">
+        <v>4100000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
         <v>4000000</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="9">
         <v>0.8</v>
       </c>
-      <c r="C11" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="13">
-        <v>0.09810000000000001</v>
-      </c>
-      <c r="E11" s="14">
-        <v>31.75</v>
-      </c>
-      <c r="F11" s="10">
-        <v>738725</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C11" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="8">
+        <v>3300000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>5000000</v>
       </c>
@@ -756,64 +643,50 @@
         <v>0.6</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="5">
+        <v>2700000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="8">
-        <v>0.0815</v>
-      </c>
-      <c r="E12" s="9">
-        <v>31.75</v>
-      </c>
-      <c r="F12" s="5">
-        <v>644007</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="15" t="s">
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="15" t="s">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="15" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="15" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -822,160 +695,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AFDC508-2E51-5A08-9B5C-3956C32DC4B9}">
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="30.7109375" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5">
-        <v>33</v>
-      </c>
-      <c r="C5" s="16">
-        <v>5043163</v>
-      </c>
-      <c r="D5" s="16">
-        <v>4202</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6">
-        <v>9</v>
-      </c>
-      <c r="C6" s="16">
-        <v>120787</v>
-      </c>
-      <c r="D6" s="16">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7">
-        <v>5</v>
-      </c>
-      <c r="C7" s="16">
-        <v>121297</v>
-      </c>
-      <c r="D7" s="16">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8">
-        <v>3</v>
-      </c>
-      <c r="C8" s="16">
-        <v>136810</v>
-      </c>
-      <c r="D8" s="16">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9">
-        <v>2</v>
-      </c>
-      <c r="C9" s="16">
-        <v>217085</v>
-      </c>
-      <c r="D9" s="16">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>34</v>
-      </c>
-      <c r="B10">
-        <v>4</v>
-      </c>
-      <c r="C10" s="16">
-        <v>49785</v>
-      </c>
-      <c r="D10" s="16">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11">
-        <v>3</v>
-      </c>
-      <c r="C11" s="16">
-        <v>16985</v>
-      </c>
-      <c r="D11" s="16">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="B12" s="15">
-        <v>59</v>
-      </c>
-      <c r="C12" s="17">
-        <v>5705913</v>
-      </c>
-      <c r="D12" s="17">
-        <v>5637</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DCFDB46-145B-5FB6-8DEC-EA73E3A2C247}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="110.7109375" customWidth="1"/>
@@ -983,42 +704,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
-        <v>38</v>
+      <c r="A3" s="12" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
-        <v>39</v>
+      <c r="A4" s="12" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="18" t="s">
-        <v>40</v>
+      <c r="A5" s="12" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
-        <v>41</v>
+      <c r="A6" s="12" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="18" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="44" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="18" t="s">
-        <v>44</v>
+      <c r="A7" s="12" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RESHIPPED (task255): keep the first $4,000,000 of each 2027 liability occurrence (loop 2, severity by coverage group)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Es2YJxT597uNAuNJZNdYR4
</commit_message>
<xml_diff>
--- a/task255/golden/retention_2027.xlsx
+++ b/task255/golden/retention_2027.xlsx
@@ -31,7 +31,7 @@
     <t>Keep the first $4,000,000 of each 2027 liability occurrence: the lowest quoted attachment the pool expects its 2027 occurrences to exceed once or less (0.8)</t>
   </si>
   <si>
-    <t>Risk financing policy 4.1 to 5.1; expected occurrences from the actuary's 85.0 law enforcement and 375.0 other occurrences above $25,000, each carried by its own ground-up severity at 2027 cost; layers of $10,000,000 above each attachment quoted by the broker on October 2, 2026.</t>
+    <t>Risk financing policy 4.1 to 5.1; expected occurrences from the actuary's 85.1 law enforcement and 347.6 other occurrences above $25,000, each carried by its own ground-up severity at 2027 cost; layers of $10,000,000 above each attachment quoted by the broker on October 2, 2026.</t>
   </si>
   <si>
     <t>Attachment per occurrence</t>
@@ -94,7 +94,7 @@
     <t>The pool's record holds an occurrence only once its member's payments reached the deductible in force on the date of the occurrence, and holds its cost only up to the pool's retention ($500,000 for 2014 to 2017, $1,000,000 from 2018); severity is fitted to that record as it came to exist.</t>
   </si>
   <si>
-    <t>Expected occurrences above an attachment: the actuary's 85.0 law enforcement occurrences above $25,000 times that severity's probability of a cost above the attachment given a cost above $25,000, plus the same for the 375.0 other occurrences (policy 4.3, Exhibit 6). Shown to one decimal; compared unrounded.</t>
+    <t>Expected occurrences above an attachment: the actuary's 85.1 law enforcement occurrences above $25,000 times that severity's probability of a cost above the attachment given a cost above $25,000, plus the same for the 347.6 other occurrences (policy 4.3, Exhibit 6). Shown to one decimal; compared unrounded.</t>
   </si>
   <si>
     <t>Expected losses to a layer: for each coverage group, its expected 2027 occurrences above $25,000 times the expected cost above the attachment, up to the $10,000,000 limit, of an occurrence costing more than $25,000 on that group's severity; rounded to the nearest hundred thousand dollars.</t>

</xml_diff>